<commit_message>
MethodMesh v1.22: refresh preset, scheduler and module contracts
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/apriltag/example_odk_showcase_apriltag_calibrate_focal.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/apriltag/example_odk_showcase_apriltag_calibrate_focal.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R62edad645c13498f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R7bab730d8602436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R07a46010cb844ac2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R81402d9c6a004d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R0fdf3b2a51ae4713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R7b86491ba67844e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,6 +301,8 @@
       <x:c r="H1" s="4" t="str">
         <x:v>intent</x:v>
       </x:c>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
@@ -313,12 +315,14 @@
         <x:v>MethodMesh — Calibrate AprilTag range</x:v>
       </x:c>
       <x:c r="D2" s="8" t="str">
-        <x:v>Measure camera-to-tag distance accurately, keep one tag front-facing, then collect stable samples in the MethodMesh live HUD before Commit.</x:v>
+        <x:v>Calibrate real-world AprilTag pose scale from a measured camera-to-tag distance. The live HUD shows raw range, variation, proposed adjustment and corrected distance before Commit.</x:v>
       </x:c>
       <x:c r="E2" s="8"/>
       <x:c r="F2" s="8"/>
       <x:c r="G2" s="8"/>
       <x:c r="H2" s="8"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -339,8 +343,10 @@
       <x:c r="F3" s="8"/>
       <x:c r="G3" s="8"/>
       <x:c r="H3" s="8" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='apriltag.calibrate_focal',input_tag_family=${tag_family},input_target_tag_id=${target_tag_id},input_tag_size_mm=${tag_size_mm},input_known_distance_mm=${known_distance_mm},input_calibration_samples=${calibration_samples},input_payload_mode='FULL',return_mode='flat')</x:v>
-      </x:c>
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='apriltag.calibrate_focal',input_tag_family=${tag_family},input_target_tag_id=${target_tag_id},input_tag_size_mm=${tag_size_mm},input_known_distance_mm=${known_distance_mm},input_calibration_samples=${calibration_samples},input_distance_scale=${distance_scale},input_payload_mode='FULL',return_mode='flat')</x:v>
+      </x:c>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="8" t="str">
@@ -363,6 +369,8 @@
         <x:v>tagStandard41h12</x:v>
       </x:c>
       <x:c r="H4" s="8"/>
+      <x:c r="I4"/>
+      <x:c r="J4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
@@ -385,6 +393,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="8"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
@@ -407,6 +417,8 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H6" s="8"/>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
@@ -429,6 +441,8 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="H7" s="8"/>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
@@ -451,39 +465,41 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="H8" s="8"/>
+      <x:c r="I8"/>
+      <x:c r="J8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>decimal</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>methodmesh_status</x:v>
+        <x:v>distance_scale</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>MethodMesh status</x:v>
+        <x:v>Distance adjustment</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>Shared transport status.</x:v>
-      </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:v>hidden-answer</x:v>
-      </x:c>
+        <x:v>Optional. Leave blank to use the saved device calibration. Corrected XYZ/range = raw pose × this value.</x:v>
+      </x:c>
+      <x:c r="E9" s="8"/>
       <x:c r="F9" s="8"/>
       <x:c r="G9" s="8"/>
       <x:c r="H9" s="8"/>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>apriltag_status</x:v>
+        <x:v>methodmesh_status</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
-        <x:v>AprilTag Status</x:v>
+        <x:v>MethodMesh status</x:v>
       </x:c>
       <x:c r="D10" s="8" t="str">
-        <x:v>Canonical capability return.</x:v>
+        <x:v>Shared transport status.</x:v>
       </x:c>
       <x:c r="E10" s="8" t="str">
         <x:v>hidden-answer</x:v>
@@ -491,16 +507,18 @@
       <x:c r="F10" s="8"/>
       <x:c r="G10" s="8"/>
       <x:c r="H10" s="8"/>
+      <x:c r="I10"/>
+      <x:c r="J10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>apriltag_result</x:v>
+        <x:v>apriltag_status</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
-        <x:v>AprilTag Result</x:v>
+        <x:v>AprilTag Status</x:v>
       </x:c>
       <x:c r="D11" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -511,16 +529,18 @@
       <x:c r="F11" s="8"/>
       <x:c r="G11" s="8"/>
       <x:c r="H11" s="8"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
-        <x:v>integer</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>apriltag_calibration_tag_id</x:v>
+        <x:v>apriltag_result</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>AprilTag Calibration Tag Id</x:v>
+        <x:v>AprilTag Result</x:v>
       </x:c>
       <x:c r="D12" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -531,16 +551,18 @@
       <x:c r="F12" s="8"/>
       <x:c r="G12" s="8"/>
       <x:c r="H12" s="8"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>apriltag_family</x:v>
+        <x:v>apriltag_calibration_tag_id</x:v>
       </x:c>
       <x:c r="C13" s="8" t="str">
-        <x:v>AprilTag Family</x:v>
+        <x:v>AprilTag Calibration Tag Id</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -551,16 +573,18 @@
       <x:c r="F13" s="8"/>
       <x:c r="G13" s="8"/>
       <x:c r="H13" s="8"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
-        <x:v>decimal</x:v>
+        <x:v>text</x:v>
       </x:c>
       <x:c r="B14" s="8" t="str">
-        <x:v>apriltag_tag_size_mm</x:v>
+        <x:v>apriltag_family</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
-        <x:v>AprilTag Tag Size Mm</x:v>
+        <x:v>AprilTag Family</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -571,16 +595,18 @@
       <x:c r="F14" s="8"/>
       <x:c r="G14" s="8"/>
       <x:c r="H14" s="8"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>apriltag_known_distance_mm</x:v>
+        <x:v>apriltag_tag_size_mm</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
-        <x:v>AprilTag Known Distance Mm</x:v>
+        <x:v>AprilTag Tag Size Mm</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -591,16 +617,18 @@
       <x:c r="F15" s="8"/>
       <x:c r="G15" s="8"/>
       <x:c r="H15" s="8"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
-        <x:v>integer</x:v>
+        <x:v>decimal</x:v>
       </x:c>
       <x:c r="B16" s="8" t="str">
-        <x:v>apriltag_calibration_sample_count</x:v>
+        <x:v>apriltag_known_distance_mm</x:v>
       </x:c>
       <x:c r="C16" s="8" t="str">
-        <x:v>AprilTag Calibration Sample Count</x:v>
+        <x:v>AprilTag Known Distance Mm</x:v>
       </x:c>
       <x:c r="D16" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -611,16 +639,18 @@
       <x:c r="F16" s="8"/>
       <x:c r="G16" s="8"/>
       <x:c r="H16" s="8"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
-        <x:v>decimal</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="B17" s="8" t="str">
-        <x:v>apriltag_mean_edge_px</x:v>
+        <x:v>apriltag_calibration_sample_count</x:v>
       </x:c>
       <x:c r="C17" s="8" t="str">
-        <x:v>AprilTag Mean Edge Px</x:v>
+        <x:v>AprilTag Calibration Sample Count</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -631,16 +661,18 @@
       <x:c r="F17" s="8"/>
       <x:c r="G17" s="8"/>
       <x:c r="H17" s="8"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B18" s="8" t="str">
-        <x:v>apriltag_edge_cv</x:v>
+        <x:v>apriltag_mean_edge_px</x:v>
       </x:c>
       <x:c r="C18" s="8" t="str">
-        <x:v>AprilTag Edge Cv</x:v>
+        <x:v>AprilTag Mean Edge Px</x:v>
       </x:c>
       <x:c r="D18" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -651,16 +683,18 @@
       <x:c r="F18" s="8"/>
       <x:c r="G18" s="8"/>
       <x:c r="H18" s="8"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str">
-        <x:v>apriltag_fx_px</x:v>
+        <x:v>apriltag_edge_cv</x:v>
       </x:c>
       <x:c r="C19" s="8" t="str">
-        <x:v>AprilTag Fx Px</x:v>
+        <x:v>AprilTag Edge Cv</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -671,16 +705,18 @@
       <x:c r="F19" s="8"/>
       <x:c r="G19" s="8"/>
       <x:c r="H19" s="8"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B20" s="8" t="str">
-        <x:v>apriltag_fy_px</x:v>
+        <x:v>apriltag_fx_px</x:v>
       </x:c>
       <x:c r="C20" s="8" t="str">
-        <x:v>AprilTag Fy Px</x:v>
+        <x:v>AprilTag Fx Px</x:v>
       </x:c>
       <x:c r="D20" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -691,16 +727,18 @@
       <x:c r="F20" s="8"/>
       <x:c r="G20" s="8"/>
       <x:c r="H20" s="8"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B21" s="8" t="str">
-        <x:v>apriltag_cx_px</x:v>
+        <x:v>apriltag_fy_px</x:v>
       </x:c>
       <x:c r="C21" s="8" t="str">
-        <x:v>AprilTag Cx Px</x:v>
+        <x:v>AprilTag Fy Px</x:v>
       </x:c>
       <x:c r="D21" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -711,16 +749,18 @@
       <x:c r="F21" s="8"/>
       <x:c r="G21" s="8"/>
       <x:c r="H21" s="8"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8" t="str">
         <x:v>decimal</x:v>
       </x:c>
       <x:c r="B22" s="8" t="str">
-        <x:v>apriltag_cy_px</x:v>
+        <x:v>apriltag_cx_px</x:v>
       </x:c>
       <x:c r="C22" s="8" t="str">
-        <x:v>AprilTag Cy Px</x:v>
+        <x:v>AprilTag Cx Px</x:v>
       </x:c>
       <x:c r="D22" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -731,16 +771,18 @@
       <x:c r="F22" s="8"/>
       <x:c r="G22" s="8"/>
       <x:c r="H22" s="8"/>
+      <x:c r="I22"/>
+      <x:c r="J22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8" t="str">
-        <x:v>integer</x:v>
+        <x:v>decimal</x:v>
       </x:c>
       <x:c r="B23" s="8" t="str">
-        <x:v>apriltag_intrinsics_width_px</x:v>
+        <x:v>apriltag_cy_px</x:v>
       </x:c>
       <x:c r="C23" s="8" t="str">
-        <x:v>AprilTag Intrinsics Width Px</x:v>
+        <x:v>AprilTag Cy Px</x:v>
       </x:c>
       <x:c r="D23" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -751,16 +793,18 @@
       <x:c r="F23" s="8"/>
       <x:c r="G23" s="8"/>
       <x:c r="H23" s="8"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8" t="str">
         <x:v>integer</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>apriltag_intrinsics_height_px</x:v>
+        <x:v>apriltag_intrinsics_width_px</x:v>
       </x:c>
       <x:c r="C24" s="8" t="str">
-        <x:v>AprilTag Intrinsics Height Px</x:v>
+        <x:v>AprilTag Intrinsics Width Px</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -771,16 +815,18 @@
       <x:c r="F24" s="8"/>
       <x:c r="G24" s="8"/>
       <x:c r="H24" s="8"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8" t="str">
-        <x:v>text</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="B25" s="8" t="str">
-        <x:v>apriltag_intrinsics_source</x:v>
+        <x:v>apriltag_intrinsics_height_px</x:v>
       </x:c>
       <x:c r="C25" s="8" t="str">
-        <x:v>AprilTag Intrinsics Source</x:v>
+        <x:v>AprilTag Intrinsics Height Px</x:v>
       </x:c>
       <x:c r="D25" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -791,16 +837,18 @@
       <x:c r="F25" s="8"/>
       <x:c r="G25" s="8"/>
       <x:c r="H25" s="8"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B26" s="8" t="str">
-        <x:v>apriltag_calibration_profile_json</x:v>
+        <x:v>apriltag_intrinsics_source</x:v>
       </x:c>
       <x:c r="C26" s="8" t="str">
-        <x:v>AprilTag Calibration Profile Json</x:v>
+        <x:v>AprilTag Intrinsics Source</x:v>
       </x:c>
       <x:c r="D26" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -811,16 +859,18 @@
       <x:c r="F26" s="8"/>
       <x:c r="G26" s="8"/>
       <x:c r="H26" s="8"/>
+      <x:c r="I26"/>
+      <x:c r="J26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B27" s="8" t="str">
-        <x:v>apriltag_geometry_valid</x:v>
+        <x:v>apriltag_calibration_profile_json</x:v>
       </x:c>
       <x:c r="C27" s="8" t="str">
-        <x:v>AprilTag Geometry Valid</x:v>
+        <x:v>AprilTag Calibration Profile Json</x:v>
       </x:c>
       <x:c r="D27" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -831,16 +881,18 @@
       <x:c r="F27" s="8"/>
       <x:c r="G27" s="8"/>
       <x:c r="H27" s="8"/>
+      <x:c r="I27"/>
+      <x:c r="J27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B28" s="8" t="str">
-        <x:v>apriltag_backend</x:v>
+        <x:v>apriltag_geometry_valid</x:v>
       </x:c>
       <x:c r="C28" s="8" t="str">
-        <x:v>AprilTag Backend</x:v>
+        <x:v>AprilTag Geometry Valid</x:v>
       </x:c>
       <x:c r="D28" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -851,16 +903,18 @@
       <x:c r="F28" s="8"/>
       <x:c r="G28" s="8"/>
       <x:c r="H28" s="8"/>
+      <x:c r="I28"/>
+      <x:c r="J28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B29" s="8" t="str">
-        <x:v>apriltag_captured_time_iso</x:v>
+        <x:v>apriltag_backend</x:v>
       </x:c>
       <x:c r="C29" s="8" t="str">
-        <x:v>AprilTag Captured Time Iso</x:v>
+        <x:v>AprilTag Backend</x:v>
       </x:c>
       <x:c r="D29" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -871,16 +925,18 @@
       <x:c r="F29" s="8"/>
       <x:c r="G29" s="8"/>
       <x:c r="H29" s="8"/>
+      <x:c r="I29"/>
+      <x:c r="J29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B30" s="8" t="str">
-        <x:v>apriltag_audit_json</x:v>
+        <x:v>apriltag_captured_time_iso</x:v>
       </x:c>
       <x:c r="C30" s="8" t="str">
-        <x:v>AprilTag Audit Json</x:v>
+        <x:v>AprilTag Captured Time Iso</x:v>
       </x:c>
       <x:c r="D30" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -891,16 +947,18 @@
       <x:c r="F30" s="8"/>
       <x:c r="G30" s="8"/>
       <x:c r="H30" s="8"/>
+      <x:c r="I30"/>
+      <x:c r="J30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B31" s="8" t="str">
-        <x:v>apriltag_warning</x:v>
+        <x:v>apriltag_audit_json</x:v>
       </x:c>
       <x:c r="C31" s="8" t="str">
-        <x:v>AprilTag Warning</x:v>
+        <x:v>AprilTag Audit Json</x:v>
       </x:c>
       <x:c r="D31" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -911,16 +969,18 @@
       <x:c r="F31" s="8"/>
       <x:c r="G31" s="8"/>
       <x:c r="H31" s="8"/>
+      <x:c r="I31"/>
+      <x:c r="J31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B32" s="8" t="str">
-        <x:v>apriltag_error</x:v>
+        <x:v>apriltag_warning</x:v>
       </x:c>
       <x:c r="C32" s="8" t="str">
-        <x:v>AprilTag Error</x:v>
+        <x:v>AprilTag Warning</x:v>
       </x:c>
       <x:c r="D32" s="8" t="str">
         <x:v>Canonical capability return.</x:v>
@@ -931,19 +991,21 @@
       <x:c r="F32" s="8"/>
       <x:c r="G32" s="8"/>
       <x:c r="H32" s="8"/>
+      <x:c r="I32"/>
+      <x:c r="J32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B33" s="8" t="str">
-        <x:v>methodmesh_full_json</x:v>
+        <x:v>apriltag_error</x:v>
       </x:c>
       <x:c r="C33" s="8" t="str">
-        <x:v>Full MethodMesh JSON</x:v>
+        <x:v>AprilTag Error</x:v>
       </x:c>
       <x:c r="D33" s="8" t="str">
-        <x:v>Complete structured/audit roundtrip return.</x:v>
+        <x:v>Canonical capability return.</x:v>
       </x:c>
       <x:c r="E33" s="8" t="str">
         <x:v>hidden-answer</x:v>
@@ -951,79 +1013,145 @@
       <x:c r="F33" s="8"/>
       <x:c r="G33" s="8"/>
       <x:c r="H33" s="8"/>
+      <x:c r="I33"/>
+      <x:c r="J33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8" t="str">
-        <x:v>end group</x:v>
-      </x:c>
-      <x:c r="B34" s="8"/>
-      <x:c r="C34" s="8"/>
-      <x:c r="D34" s="8"/>
-      <x:c r="E34" s="8"/>
+        <x:v>decimal</x:v>
+      </x:c>
+      <x:c r="B34" s="8" t="str">
+        <x:v>apriltag_distance_scale</x:v>
+      </x:c>
+      <x:c r="C34" s="8" t="str">
+        <x:v>AprilTag Distance Scale</x:v>
+      </x:c>
+      <x:c r="D34" s="8" t="str">
+        <x:v>Canonical capability return.</x:v>
+      </x:c>
+      <x:c r="E34" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F34" s="8"/>
       <x:c r="G34" s="8"/>
       <x:c r="H34" s="8"/>
+      <x:c r="I34"/>
+      <x:c r="J34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8" t="str">
-        <x:v>note</x:v>
+        <x:v>decimal</x:v>
       </x:c>
       <x:c r="B35" s="8" t="str">
-        <x:v>return_summary</x:v>
+        <x:v>apriltag_raw_distance_m</x:v>
       </x:c>
       <x:c r="C35" s="8" t="str">
-        <x:v>MethodMesh result captured</x:v>
+        <x:v>AprilTag Raw Distance M</x:v>
       </x:c>
       <x:c r="D35" s="8" t="str">
-        <x:v>Continue the study form.</x:v>
-      </x:c>
-      <x:c r="E35" s="8"/>
+        <x:v>Canonical capability return.</x:v>
+      </x:c>
+      <x:c r="E35" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F35" s="8"/>
       <x:c r="G35" s="8"/>
       <x:c r="H35" s="8"/>
+      <x:c r="I35"/>
+      <x:c r="J35"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="8"/>
-      <x:c r="B36" s="8"/>
-      <x:c r="C36" s="8"/>
-      <x:c r="D36" s="8"/>
-      <x:c r="E36" s="8"/>
+      <x:c r="A36" s="8" t="str">
+        <x:v>decimal</x:v>
+      </x:c>
+      <x:c r="B36" s="8" t="str">
+        <x:v>apriltag_corrected_distance_m</x:v>
+      </x:c>
+      <x:c r="C36" s="8" t="str">
+        <x:v>AprilTag Corrected Distance M</x:v>
+      </x:c>
+      <x:c r="D36" s="8" t="str">
+        <x:v>Canonical capability return.</x:v>
+      </x:c>
+      <x:c r="E36" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F36" s="8"/>
       <x:c r="G36" s="8"/>
       <x:c r="H36" s="8"/>
+      <x:c r="I36"/>
+      <x:c r="J36"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="8"/>
-      <x:c r="B37" s="8"/>
-      <x:c r="C37" s="8"/>
-      <x:c r="D37" s="8"/>
-      <x:c r="E37" s="8"/>
+      <x:c r="A37" s="8" t="str">
+        <x:v>decimal</x:v>
+      </x:c>
+      <x:c r="B37" s="8" t="str">
+        <x:v>apriltag_effective_tag_size_mm</x:v>
+      </x:c>
+      <x:c r="C37" s="8" t="str">
+        <x:v>AprilTag Effective Tag Size Mm</x:v>
+      </x:c>
+      <x:c r="D37" s="8" t="str">
+        <x:v>Canonical capability return.</x:v>
+      </x:c>
+      <x:c r="E37" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F37" s="8"/>
       <x:c r="G37" s="8"/>
       <x:c r="H37" s="8"/>
+      <x:c r="I37"/>
+      <x:c r="J37"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="8"/>
-      <x:c r="B38" s="8"/>
-      <x:c r="C38" s="8"/>
-      <x:c r="D38" s="8"/>
-      <x:c r="E38" s="8"/>
+      <x:c r="A38" s="8" t="str">
+        <x:v>decimal</x:v>
+      </x:c>
+      <x:c r="B38" s="8" t="str">
+        <x:v>apriltag_range_cv</x:v>
+      </x:c>
+      <x:c r="C38" s="8" t="str">
+        <x:v>AprilTag Range Cv</x:v>
+      </x:c>
+      <x:c r="D38" s="8" t="str">
+        <x:v>Canonical capability return.</x:v>
+      </x:c>
+      <x:c r="E38" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F38" s="8"/>
       <x:c r="G38" s="8"/>
       <x:c r="H38" s="8"/>
+      <x:c r="I38"/>
+      <x:c r="J38"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="8"/>
-      <x:c r="B39" s="8"/>
-      <x:c r="C39" s="8"/>
-      <x:c r="D39" s="8"/>
-      <x:c r="E39" s="8"/>
+      <x:c r="A39" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B39" s="8" t="str">
+        <x:v>methodmesh_full_json</x:v>
+      </x:c>
+      <x:c r="C39" s="8" t="str">
+        <x:v>Full MethodMesh JSON</x:v>
+      </x:c>
+      <x:c r="D39" s="8" t="str">
+        <x:v>Complete structured/audit roundtrip return.</x:v>
+      </x:c>
+      <x:c r="E39" s="8" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
       <x:c r="F39" s="8"/>
       <x:c r="G39" s="8"/>
       <x:c r="H39" s="8"/>
+      <x:c r="I39"/>
+      <x:c r="J39"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="8"/>
+      <x:c r="A40" s="8" t="str">
+        <x:v>end group</x:v>
+      </x:c>
       <x:c r="B40" s="8"/>
       <x:c r="C40" s="8"/>
       <x:c r="D40" s="8"/>
@@ -1031,16 +1159,28 @@
       <x:c r="F40" s="8"/>
       <x:c r="G40" s="8"/>
       <x:c r="H40" s="8"/>
+      <x:c r="I40"/>
+      <x:c r="J40"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="8"/>
-      <x:c r="B41" s="8"/>
-      <x:c r="C41" s="8"/>
-      <x:c r="D41" s="8"/>
+      <x:c r="A41" s="8" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="B41" s="8" t="str">
+        <x:v>return_summary</x:v>
+      </x:c>
+      <x:c r="C41" s="8" t="str">
+        <x:v>MethodMesh result captured</x:v>
+      </x:c>
+      <x:c r="D41" s="8" t="str">
+        <x:v>Continue the study form.</x:v>
+      </x:c>
       <x:c r="E41" s="8"/>
       <x:c r="F41" s="8"/>
       <x:c r="G41" s="8"/>
       <x:c r="H41" s="8"/>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="8"/>

</xml_diff>